<commit_message>
resultats minsup ESBL 2019-2021
</commit_message>
<xml_diff>
--- a/results_minsup_ESBL/minsup_0_001/rep1/describ_graphs_0.95.xlsx
+++ b/results_minsup_ESBL/minsup_0_001/rep1/describ_graphs_0.95.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">dataset</t>
   </si>
@@ -26,7 +26,31 @@
     <t xml:space="preserve">2018_BLSE</t>
   </si>
   <si>
+    <t xml:space="preserve">2019_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021_BLSE</t>
+  </si>
+  <si>
     <t xml:space="preserve">2022_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2022_non_BLSE</t>
   </si>
 </sst>
 </file>
@@ -371,10 +395,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>11</v>
+        <v>10.5925925925926</v>
       </c>
       <c r="C2" t="n">
-        <v>0.44</v>
+        <v>0.407407407407407</v>
       </c>
     </row>
     <row r="3">
@@ -382,10 +406,98 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>12.2222222222222</v>
       </c>
       <c r="C3" t="n">
-        <v>0.52</v>
+        <v>0.47008547008547</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>12.5925925925926</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.484330484330484</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>12.5185185185185</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.481481481481482</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="n">
+        <v>12.5185185185185</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.481481481481482</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1.92592592592593</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0740740740740741</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2.37037037037037</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0911680911680912</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2.2962962962963</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0883190883190883</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2.51851851851852</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0968660968660969</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2.59259259259259</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0997150997150997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>